<commit_message>
data(legacy-pilot06): populate wave 1 evidence
Phase 5C: research and populate evidence-backed DESTINATIONS identity/geography and CLIMATE_MONTHLY (12 rows each) for the two Wave 1 legacy-migration-pilot-06 destinations (The Hague, Kyoto), citing KNMI, JMA, CBS, City of Kyoto, and official municipal/tourism sources. The other 4 pilot destinations remain untouched identity-only skeletons. Adds a per-destination research ledger with full provenance and an explicit notResearchedThisPass list; extends the structural validator with source-backed-population + cross-destination-isolation checks; extends the real deterministic-parser test suite (7 tests) proving isolation in both directions. No Supabase write. No change to any of the 8 other tracked .xlsx workbooks (SHA-256 verified).
</commit_message>
<xml_diff>
--- a/data/legacy-migration-pilot-06/DestinationFinderAI_LegacyMigrationPilot06_v3.3_SKELETON.xlsx
+++ b/data/legacy-migration-pilot-06/DestinationFinderAI_LegacyMigrationPilot06_v3.3_SKELETON.xlsx
@@ -854,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -921,6 +921,1002 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>70</v>
+      </c>
+      <c r="F2" t="n">
+        <v>86</v>
+      </c>
+      <c r="G2" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>84</v>
+      </c>
+      <c r="G3" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="F4" t="n">
+        <v>83</v>
+      </c>
+      <c r="G4" t="n">
+        <v>152</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>79</v>
+      </c>
+      <c r="G5" t="n">
+        <v>207.2</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>78</v>
+      </c>
+      <c r="G6" t="n">
+        <v>240.5</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>79</v>
+      </c>
+      <c r="G7" t="n">
+        <v>229.3</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="F8" t="n">
+        <v>80</v>
+      </c>
+      <c r="G8" t="n">
+        <v>237.5</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="D9" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>84</v>
+      </c>
+      <c r="F9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" t="n">
+        <v>213.4</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>83</v>
+      </c>
+      <c r="G10" t="n">
+        <v>160</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="F11" t="n">
+        <v>84</v>
+      </c>
+      <c r="G11" t="n">
+        <v>116.7</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="F12" t="n">
+        <v>87</v>
+      </c>
+      <c r="G12" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>87</v>
+      </c>
+      <c r="G13" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>67</v>
+      </c>
+      <c r="G14" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="H14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E15" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>65</v>
+      </c>
+      <c r="G15" t="n">
+        <v>122.2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>61</v>
+      </c>
+      <c r="G16" t="n">
+        <v>155.4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E17" t="n">
+        <v>117</v>
+      </c>
+      <c r="F17" t="n">
+        <v>59</v>
+      </c>
+      <c r="G17" t="n">
+        <v>177.3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E18" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="F18" t="n">
+        <v>60</v>
+      </c>
+      <c r="G18" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>199.7</v>
+      </c>
+      <c r="F19" t="n">
+        <v>66</v>
+      </c>
+      <c r="G19" t="n">
+        <v>133.1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>32</v>
+      </c>
+      <c r="D20" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="E20" t="n">
+        <v>223.6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>69</v>
+      </c>
+      <c r="G20" t="n">
+        <v>142.7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>153.8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>66</v>
+      </c>
+      <c r="G21" t="n">
+        <v>182.7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>9</v>
+      </c>
+      <c r="C22" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>67</v>
+      </c>
+      <c r="G22" t="n">
+        <v>142.7</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D23" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>143.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>68</v>
+      </c>
+      <c r="G23" t="n">
+        <v>156</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>11</v>
+      </c>
+      <c r="C24" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="F24" t="n">
+        <v>68</v>
+      </c>
+      <c r="G24" t="n">
+        <v>140.7</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>68</v>
+      </c>
+      <c r="G25" t="n">
+        <v>134.4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -4741,7 +5737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4793,6 +5789,339 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands__source_1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Royal Netherlands Meteorological Institute (KNMI), Valkenburg station, 1981-2010 normal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20171010161642/http://www.klimaatatlas.nl/tabel/stationsdata/klimtab_8110_210.pdf</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>official_climate_normal</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>kyoto-japan__source_2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Japan Meteorological Agency (JMA), station block_no 47759, 1991-2020 normal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.data.jma.go.jp/obd/stats/etrn/index.php?prec_no=61&amp;block_no=47759&amp;year=&amp;month=&amp;day=&amp;view=</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>official_climate_normal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands__source_3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Wikipedia (The Hague) infobox, citing the municipality's own administrative status</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/The_Hague</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands__source_4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Statistics Netherlands (CBS), via Wikipedia infobox citation</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://opendata.cbs.nl/statline/#/CBS/en/dataset/37259eng/table</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands__source_5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Netherlands is a Eurozone member state (uncontroversial, well-established national fact)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.government.nl/topics/immigration-to-the-netherlands</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands__source_6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Municipality of The Hague official website (confirmed live and reachable this session)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.denhaag.nl/en/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>kyoto-japan__source_7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Wikipedia (Kyoto) infobox</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Kyoto</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>kyoto-japan__source_8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>City of Kyoto, Estimated Population (推計人口), via Wikipedia infobox citation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www2.city.kyoto.lg.jp/sogo/toukei/Population/Suikei/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>kyoto-japan__source_9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Kyoto City Official Travel Guide - City of Kyoto and Kyoto City Tourism Association</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://kyoto.travel/en/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>research_citation</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -10267,7 +11596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10470,7 +11799,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Skeleton package creation date</t>
+          <t>Phase 5C update date</t>
         </is>
       </c>
     </row>
@@ -10482,12 +11811,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>empty_skeleton_pending_research</t>
+          <t>wave1_evidence_backed_partial</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No destination content has been researched or populated yet</t>
+          <t>The Hague and Kyoto have evidence-backed DESTINATIONS identity/geography + CLIMATE_MONTHLY fields; the other 4 destinations remain an empty identity skeleton</t>
         </is>
       </c>
     </row>
@@ -10516,12 +11845,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PHASE_5A_IDENTITY_SKELETON</t>
+          <t>PHASE_5C_WAVE1_EVIDENCE_POPULATION</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Structural identity + empty content sheets only; see pilot-manifest.json for status</t>
+          <t>Wave 1 (The Hague, Kyoto) identity/geography/climate populated from cited sources; see pilot-manifest.json and research-ledger/ for provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>wave1_researched_keys</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>the-hague-netherlands; kyoto-japan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Only these destination_keys received Phase 5C content population</t>
         </is>
       </c>
     </row>
@@ -10536,7 +11882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10578,6 +11924,28 @@
         </is>
       </c>
       <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3.3-pilot06-phase5c</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Populated evidence-backed DESTINATIONS identity/geography and CLIMATE_MONTHLY (12 rows each) for The Hague and Kyoto (Wave 1), citing KNMI/JMA/CBS/City of Kyoto/Wikipedia-relayed-official-sources; added SOURCES rows.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The other 4 pilot destinations remain untouched, identity-only skeletons. See research-ledger/ for full provenance and notResearchedThisPass fields.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
@@ -10652,7 +12020,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
+          <t>PARTIAL (identity + climate only)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10677,7 +12045,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PRE_MIGRATION_NOT_YET_RESEARCHED</t>
+          <t>WAVE1_IDENTITY_AND_CLIMATE_RESEARCHED</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -10699,7 +12067,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
+          <t>PARTIAL (identity + climate only)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10724,7 +12092,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>PRE_MIGRATION_NOT_YET_RESEARCHED</t>
+          <t>WAVE1_IDENTITY_AND_CLIMATE_RESEARCHED</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -11613,9 +12981,61 @@
           <t>Netherlands</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>South Holland</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>the-hague-netherlands</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Europe/Amsterdam</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>549163</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Rotterdam-The Hague metropolitan area (2,390,101, CBS/COROP, 1 Jan 2021)</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>https://www.denhaag.nl/en/</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Hague%2C+Netherlands</t>
         </is>
       </c>
     </row>
@@ -11635,9 +13055,58 @@
           <t>Japan</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kyoto Prefecture</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>kyoto-japan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Asia/Tokyo</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1431419</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Greater Kyoto metropolitan area (3,783,014, Japan Statistics Bureau)</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>35.01</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>135.77</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>https://kyoto.travel/en/</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Kyoto%2C+Japan</t>
         </is>
       </c>
     </row>

</xml_diff>